<commit_message>
feat: Implement Stock Inbound and Outbound Management
- Added StockInbound and StockInboundDetail models for managing inbound stock.
- Created StockMovement and StockOutbound models for tracking stock movements and outbound processes.
- Developed StockOutboundDetail model to handle details of outbound stock.
- Updated MasterBarangModel to remove loc_id and include qty_kg.
- Modified TempUploadModel to change the table name for temporary uploads.
- Created migration files for new stock management tables including wrm_stock_inbound, wrm_stock_outbound, and their respective details.
- Updated sidebar permissions and routes to reflect new inventory management structure.
- Refactored views for stock management, including index and outbound views, to support new functionality.
- Removed obsolete transfer view and associated logic.
</commit_message>
<xml_diff>
--- a/public/assets/templates/excel/template_stock_gula_wrm.xlsx
+++ b/public/assets/templates/excel/template_stock_gula_wrm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\project_warehouse\public\assets\templates\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81B1E89-E422-4F87-9CF0-3394D40B8810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B8615E9-06B5-49FC-8717-206E60346A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>BARCODE</t>
   </si>
@@ -37,10 +37,22 @@
     <t>SUPPLIER</t>
   </si>
   <si>
+    <t>PALLET</t>
+  </si>
+  <si>
+    <t>MATERAL DESCRIPTION</t>
+  </si>
+  <si>
+    <t>PLANT</t>
+  </si>
+  <si>
+    <t>S_LOC</t>
+  </si>
+  <si>
+    <t>UOM</t>
+  </si>
+  <si>
     <t>STATUS</t>
-  </si>
-  <si>
-    <t>PALLET</t>
   </si>
   <si>
     <t>CATATAN</t>
@@ -109,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -124,6 +136,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,61 +441,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" s="2" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="K1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>7</v>
+      <c r="L1" s="7" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
+      <c r="B2" s="5"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
     </row>
-    <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="5"/>
-      <c r="B3" s="6"/>
+      <c r="B3" s="5"/>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>